<commit_message>
Update dark mode charts and UI improvements
</commit_message>
<xml_diff>
--- a/static/annuitySchedule_results.xlsx
+++ b/static/annuitySchedule_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -440,13 +440,13 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B2" t="n">
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>16136829</v>
+        <v>35024487</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -454,324 +454,352 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B3" t="n">
-        <v>1452314</v>
+        <v>3852693</v>
       </c>
       <c r="C3" t="n">
-        <v>16624275</v>
+        <v>36284015</v>
       </c>
       <c r="D3" t="n">
-        <v>964868</v>
+        <v>2593165</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B4" t="n">
-        <v>1496184</v>
+        <v>3991241</v>
       </c>
       <c r="C4" t="n">
-        <v>17107348</v>
+        <v>37552433</v>
       </c>
       <c r="D4" t="n">
-        <v>1013111</v>
+        <v>2722823</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B5" t="n">
-        <v>1539661</v>
+        <v>4130767</v>
       </c>
       <c r="C5" t="n">
-        <v>17583243</v>
+        <v>38824236</v>
       </c>
       <c r="D5" t="n">
-        <v>1063766</v>
+        <v>2858964</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B6" t="n">
-        <v>1582491</v>
+        <v>4270665</v>
       </c>
       <c r="C6" t="n">
-        <v>18048779</v>
+        <v>40092989</v>
       </c>
       <c r="D6" t="n">
-        <v>1116955</v>
+        <v>3001912</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B7" t="n">
-        <v>1624390</v>
+        <v>4410228</v>
       </c>
       <c r="C7" t="n">
-        <v>18500366</v>
+        <v>41351209</v>
       </c>
       <c r="D7" t="n">
-        <v>1172803</v>
+        <v>3152008</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B8" t="n">
-        <v>1665032</v>
+        <v>4548632</v>
       </c>
       <c r="C8" t="n">
-        <v>18933955</v>
+        <v>42590233</v>
       </c>
       <c r="D8" t="n">
-        <v>1231443</v>
+        <v>3309608</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B9" t="n">
-        <v>1704055</v>
+        <v>4684925</v>
       </c>
       <c r="C9" t="n">
-        <v>19344995</v>
+        <v>43800069</v>
       </c>
       <c r="D9" t="n">
-        <v>1293015</v>
+        <v>3475089</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B10" t="n">
-        <v>1741049</v>
+        <v>4818007</v>
       </c>
       <c r="C10" t="n">
-        <v>19728378</v>
+        <v>44969233</v>
       </c>
       <c r="D10" t="n">
-        <v>1357666</v>
+        <v>3648843</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B11" t="n">
-        <v>1775554</v>
+        <v>4946615</v>
       </c>
       <c r="C11" t="n">
-        <v>20078383</v>
+        <v>46084563</v>
       </c>
       <c r="D11" t="n">
-        <v>1425549</v>
+        <v>3831285</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B12" t="n">
-        <v>1807054</v>
+        <v>5069301</v>
       </c>
       <c r="C12" t="n">
-        <v>20388611</v>
+        <v>47131014</v>
       </c>
       <c r="D12" t="n">
-        <v>1496826</v>
+        <v>4022850</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B13" t="n">
-        <v>1834974</v>
+        <v>5184411</v>
       </c>
       <c r="C13" t="n">
-        <v>20651917</v>
+        <v>48091433</v>
       </c>
       <c r="D13" t="n">
-        <v>1571668</v>
+        <v>4223992</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B14" t="n">
-        <v>1858672</v>
+        <v>5290057</v>
       </c>
       <c r="C14" t="n">
-        <v>20860338</v>
+        <v>48946298</v>
       </c>
       <c r="D14" t="n">
-        <v>1650251</v>
+        <v>4435192</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B15" t="n">
-        <v>1877430</v>
+        <v>5384092</v>
       </c>
       <c r="C15" t="n">
-        <v>21005004</v>
+        <v>49673439</v>
       </c>
       <c r="D15" t="n">
-        <v>1732764</v>
+        <v>4656951</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B16" t="n">
-        <v>1890450</v>
+        <v>5464078</v>
       </c>
       <c r="C16" t="n">
-        <v>21076052</v>
+        <v>50247718</v>
       </c>
       <c r="D16" t="n">
-        <v>1819402</v>
+        <v>4889799</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B17" t="n">
-        <v>1896844</v>
+        <v>5527248</v>
       </c>
       <c r="C17" t="n">
-        <v>21062524</v>
+        <v>50640677</v>
       </c>
       <c r="D17" t="n">
-        <v>1910372</v>
+        <v>5134289</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B18" t="n">
-        <v>1895627</v>
+        <v>5570474</v>
       </c>
       <c r="C18" t="n">
-        <v>20952260</v>
+        <v>50820148</v>
       </c>
       <c r="D18" t="n">
-        <v>2005891</v>
+        <v>5391003</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B19" t="n">
-        <v>1885703</v>
+        <v>5590216</v>
       </c>
       <c r="C19" t="n">
-        <v>20731778</v>
+        <v>50749811</v>
       </c>
       <c r="D19" t="n">
-        <v>2106185</v>
+        <v>5660553</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B20" t="n">
-        <v>1865860</v>
+        <v>5582479</v>
       </c>
       <c r="C20" t="n">
-        <v>20386143</v>
+        <v>50388709</v>
       </c>
       <c r="D20" t="n">
-        <v>2211495</v>
+        <v>5943581</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B21" t="n">
-        <v>1834752</v>
+        <v>5542757</v>
       </c>
       <c r="C21" t="n">
-        <v>19898826</v>
+        <v>49690706</v>
       </c>
       <c r="D21" t="n">
-        <v>2322069</v>
+        <v>6240760</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B22" t="n">
-        <v>1790894</v>
+        <v>5465977</v>
       </c>
       <c r="C22" t="n">
-        <v>19251547</v>
+        <v>48603885</v>
       </c>
       <c r="D22" t="n">
-        <v>2438173</v>
+        <v>6552798</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B23" t="n">
-        <v>1732639</v>
+        <v>5346427</v>
       </c>
       <c r="C23" t="n">
-        <v>18424104</v>
+        <v>47069874</v>
       </c>
       <c r="D23" t="n">
-        <v>2560082</v>
+        <v>6880438</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B24" t="n">
-        <v>1658169</v>
+        <v>5177686</v>
       </c>
       <c r="C24" t="n">
-        <v>17394187</v>
+        <v>45023100</v>
       </c>
       <c r="D24" t="n">
-        <v>2688086</v>
+        <v>7224460</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
+        <v>83</v>
+      </c>
+      <c r="B25" t="n">
+        <v>4952541</v>
+      </c>
+      <c r="C25" t="n">
+        <v>42389958</v>
+      </c>
+      <c r="D25" t="n">
+        <v>7585683</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>84</v>
+      </c>
+      <c r="B26" t="n">
+        <v>4662895</v>
+      </c>
+      <c r="C26" t="n">
+        <v>39087886</v>
+      </c>
+      <c r="D26" t="n">
+        <v>7964967</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
         <v>85</v>
       </c>
-      <c r="B25" t="n">
-        <v>1565476</v>
-      </c>
-      <c r="C25" t="n">
-        <v>16137173</v>
-      </c>
-      <c r="D25" t="n">
-        <v>2822490</v>
+      <c r="B27" t="n">
+        <v>4299667</v>
+      </c>
+      <c r="C27" t="n">
+        <v>35024337</v>
+      </c>
+      <c r="D27" t="n">
+        <v>8363216</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rectifed issues with calculators
</commit_message>
<xml_diff>
--- a/static/annuitySchedule_results.xlsx
+++ b/static/annuitySchedule_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -440,13 +440,13 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="B2" t="n">
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>35024487</v>
+        <v>6539011</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -454,352 +454,674 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="B3" t="n">
-        <v>3852693</v>
+        <v>980851</v>
       </c>
       <c r="C3" t="n">
-        <v>36284015</v>
+        <v>6858362</v>
       </c>
       <c r="D3" t="n">
-        <v>2593165</v>
+        <v>661500</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>62</v>
+        <v>34</v>
       </c>
       <c r="B4" t="n">
-        <v>3991241</v>
+        <v>1028754</v>
       </c>
       <c r="C4" t="n">
-        <v>37552433</v>
+        <v>7192541</v>
       </c>
       <c r="D4" t="n">
-        <v>2722823</v>
+        <v>694575</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>63</v>
+        <v>35</v>
       </c>
       <c r="B5" t="n">
-        <v>4130767</v>
+        <v>1078881</v>
       </c>
       <c r="C5" t="n">
-        <v>38824236</v>
+        <v>7542119</v>
       </c>
       <c r="D5" t="n">
-        <v>2858964</v>
+        <v>729303</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>64</v>
+        <v>36</v>
       </c>
       <c r="B6" t="n">
-        <v>4270665</v>
+        <v>1131317</v>
       </c>
       <c r="C6" t="n">
-        <v>40092989</v>
+        <v>7907668</v>
       </c>
       <c r="D6" t="n">
-        <v>3001912</v>
+        <v>765768</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>65</v>
+        <v>37</v>
       </c>
       <c r="B7" t="n">
-        <v>4410228</v>
+        <v>1186150</v>
       </c>
       <c r="C7" t="n">
-        <v>41351209</v>
+        <v>8289761</v>
       </c>
       <c r="D7" t="n">
-        <v>3152008</v>
+        <v>804057</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>66</v>
+        <v>38</v>
       </c>
       <c r="B8" t="n">
-        <v>4548632</v>
+        <v>1243464</v>
       </c>
       <c r="C8" t="n">
-        <v>42590233</v>
+        <v>8688965</v>
       </c>
       <c r="D8" t="n">
-        <v>3309608</v>
+        <v>844260</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>67</v>
+        <v>39</v>
       </c>
       <c r="B9" t="n">
-        <v>4684925</v>
+        <v>1303344</v>
       </c>
       <c r="C9" t="n">
-        <v>43800069</v>
+        <v>9105836</v>
       </c>
       <c r="D9" t="n">
-        <v>3475089</v>
+        <v>886473</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>68</v>
+        <v>40</v>
       </c>
       <c r="B10" t="n">
-        <v>4818007</v>
+        <v>1365875</v>
       </c>
       <c r="C10" t="n">
-        <v>44969233</v>
+        <v>9540915</v>
       </c>
       <c r="D10" t="n">
-        <v>3648843</v>
+        <v>930796</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>69</v>
+        <v>41</v>
       </c>
       <c r="B11" t="n">
-        <v>4946615</v>
+        <v>1431137</v>
       </c>
       <c r="C11" t="n">
-        <v>46084563</v>
+        <v>9994716</v>
       </c>
       <c r="D11" t="n">
-        <v>3831285</v>
+        <v>977336</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>70</v>
+        <v>42</v>
       </c>
       <c r="B12" t="n">
-        <v>5069301</v>
+        <v>1499207</v>
       </c>
       <c r="C12" t="n">
-        <v>47131014</v>
+        <v>10467720</v>
       </c>
       <c r="D12" t="n">
-        <v>4022850</v>
+        <v>1026203</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>71</v>
+        <v>43</v>
       </c>
       <c r="B13" t="n">
-        <v>5184411</v>
+        <v>1570158</v>
       </c>
       <c r="C13" t="n">
-        <v>48091433</v>
+        <v>10960365</v>
       </c>
       <c r="D13" t="n">
-        <v>4223992</v>
+        <v>1077513</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>72</v>
+        <v>44</v>
       </c>
       <c r="B14" t="n">
-        <v>5290057</v>
+        <v>1644054</v>
       </c>
       <c r="C14" t="n">
-        <v>48946298</v>
+        <v>11473030</v>
       </c>
       <c r="D14" t="n">
-        <v>4435192</v>
+        <v>1131389</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="B15" t="n">
-        <v>5384092</v>
+        <v>1720954</v>
       </c>
       <c r="C15" t="n">
-        <v>49673439</v>
+        <v>12006026</v>
       </c>
       <c r="D15" t="n">
-        <v>4656951</v>
+        <v>1187958</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>74</v>
+        <v>46</v>
       </c>
       <c r="B16" t="n">
-        <v>5464078</v>
+        <v>1800903</v>
       </c>
       <c r="C16" t="n">
-        <v>50247718</v>
+        <v>12559573</v>
       </c>
       <c r="D16" t="n">
-        <v>4889799</v>
+        <v>1247356</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="B17" t="n">
-        <v>5527248</v>
+        <v>1883935</v>
       </c>
       <c r="C17" t="n">
-        <v>50640677</v>
+        <v>13133784</v>
       </c>
       <c r="D17" t="n">
-        <v>5134289</v>
+        <v>1309724</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="B18" t="n">
-        <v>5570474</v>
+        <v>1970067</v>
       </c>
       <c r="C18" t="n">
-        <v>50820148</v>
+        <v>13728641</v>
       </c>
       <c r="D18" t="n">
-        <v>5391003</v>
+        <v>1375210</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>77</v>
+        <v>49</v>
       </c>
       <c r="B19" t="n">
-        <v>5590216</v>
+        <v>2059296</v>
       </c>
       <c r="C19" t="n">
-        <v>50749811</v>
+        <v>14343966</v>
       </c>
       <c r="D19" t="n">
-        <v>5660553</v>
+        <v>1443971</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>78</v>
+        <v>50</v>
       </c>
       <c r="B20" t="n">
-        <v>5582479</v>
+        <v>2151594</v>
       </c>
       <c r="C20" t="n">
-        <v>50388709</v>
+        <v>14979390</v>
       </c>
       <c r="D20" t="n">
-        <v>5943581</v>
+        <v>1516170</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>79</v>
+        <v>51</v>
       </c>
       <c r="B21" t="n">
-        <v>5542757</v>
+        <v>2246908</v>
       </c>
       <c r="C21" t="n">
-        <v>49690706</v>
+        <v>15634320</v>
       </c>
       <c r="D21" t="n">
-        <v>6240760</v>
+        <v>1591978</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>80</v>
+        <v>52</v>
       </c>
       <c r="B22" t="n">
-        <v>5465977</v>
+        <v>2345148</v>
       </c>
       <c r="C22" t="n">
-        <v>48603885</v>
+        <v>16307891</v>
       </c>
       <c r="D22" t="n">
-        <v>6552798</v>
+        <v>1671577</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>81</v>
+        <v>53</v>
       </c>
       <c r="B23" t="n">
-        <v>5346427</v>
+        <v>2446183</v>
       </c>
       <c r="C23" t="n">
-        <v>47069874</v>
+        <v>16998918</v>
       </c>
       <c r="D23" t="n">
-        <v>6880438</v>
+        <v>1755156</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>82</v>
+        <v>54</v>
       </c>
       <c r="B24" t="n">
-        <v>5177686</v>
+        <v>2549837</v>
       </c>
       <c r="C24" t="n">
-        <v>45023100</v>
+        <v>17705841</v>
       </c>
       <c r="D24" t="n">
-        <v>7224460</v>
+        <v>1842914</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>83</v>
+        <v>55</v>
       </c>
       <c r="B25" t="n">
-        <v>4952541</v>
+        <v>2655876</v>
       </c>
       <c r="C25" t="n">
-        <v>42389958</v>
+        <v>18426658</v>
       </c>
       <c r="D25" t="n">
-        <v>7585683</v>
+        <v>1935059</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="B26" t="n">
-        <v>4662895</v>
+        <v>2763998</v>
       </c>
       <c r="C26" t="n">
-        <v>39087886</v>
+        <v>19158844</v>
       </c>
       <c r="D26" t="n">
-        <v>7964967</v>
+        <v>2031812</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>85</v>
+        <v>57</v>
       </c>
       <c r="B27" t="n">
-        <v>4299667</v>
+        <v>2873826</v>
       </c>
       <c r="C27" t="n">
-        <v>35024337</v>
+        <v>19899267</v>
       </c>
       <c r="D27" t="n">
-        <v>8363216</v>
+        <v>2133403</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>58</v>
+      </c>
+      <c r="B28" t="n">
+        <v>2984890</v>
+      </c>
+      <c r="C28" t="n">
+        <v>20644084</v>
+      </c>
+      <c r="D28" t="n">
+        <v>2240073</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>59</v>
+      </c>
+      <c r="B29" t="n">
+        <v>3096612</v>
+      </c>
+      <c r="C29" t="n">
+        <v>21388619</v>
+      </c>
+      <c r="D29" t="n">
+        <v>2352077</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>60</v>
+      </c>
+      <c r="B30" t="n">
+        <v>3208292</v>
+      </c>
+      <c r="C30" t="n">
+        <v>22127230</v>
+      </c>
+      <c r="D30" t="n">
+        <v>2469681</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>61</v>
+      </c>
+      <c r="B31" t="n">
+        <v>3319084</v>
+      </c>
+      <c r="C31" t="n">
+        <v>22853149</v>
+      </c>
+      <c r="D31" t="n">
+        <v>2593165</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>62</v>
+      </c>
+      <c r="B32" t="n">
+        <v>3427972</v>
+      </c>
+      <c r="C32" t="n">
+        <v>23558298</v>
+      </c>
+      <c r="D32" t="n">
+        <v>2722823</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>63</v>
+      </c>
+      <c r="B33" t="n">
+        <v>3533744</v>
+      </c>
+      <c r="C33" t="n">
+        <v>24233078</v>
+      </c>
+      <c r="D33" t="n">
+        <v>2858964</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>64</v>
+      </c>
+      <c r="B34" t="n">
+        <v>3634961</v>
+      </c>
+      <c r="C34" t="n">
+        <v>24866126</v>
+      </c>
+      <c r="D34" t="n">
+        <v>3001913</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>65</v>
+      </c>
+      <c r="B35" t="n">
+        <v>3729918</v>
+      </c>
+      <c r="C35" t="n">
+        <v>25444036</v>
+      </c>
+      <c r="D35" t="n">
+        <v>3152008</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>66</v>
+      </c>
+      <c r="B36" t="n">
+        <v>3816605</v>
+      </c>
+      <c r="C36" t="n">
+        <v>25951032</v>
+      </c>
+      <c r="D36" t="n">
+        <v>3309609</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>67</v>
+      </c>
+      <c r="B37" t="n">
+        <v>3892654</v>
+      </c>
+      <c r="C37" t="n">
+        <v>26368597</v>
+      </c>
+      <c r="D37" t="n">
+        <v>3475089</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>68</v>
+      </c>
+      <c r="B38" t="n">
+        <v>3955289</v>
+      </c>
+      <c r="C38" t="n">
+        <v>26675042</v>
+      </c>
+      <c r="D38" t="n">
+        <v>3648844</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>69</v>
+      </c>
+      <c r="B39" t="n">
+        <v>4001256</v>
+      </c>
+      <c r="C39" t="n">
+        <v>26845012</v>
+      </c>
+      <c r="D39" t="n">
+        <v>3831286</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>70</v>
+      </c>
+      <c r="B40" t="n">
+        <v>4026751</v>
+      </c>
+      <c r="C40" t="n">
+        <v>26848913</v>
+      </c>
+      <c r="D40" t="n">
+        <v>4022850</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>71</v>
+      </c>
+      <c r="B41" t="n">
+        <v>4027336</v>
+      </c>
+      <c r="C41" t="n">
+        <v>26652256</v>
+      </c>
+      <c r="D41" t="n">
+        <v>4223993</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>72</v>
+      </c>
+      <c r="B42" t="n">
+        <v>3997838</v>
+      </c>
+      <c r="C42" t="n">
+        <v>26214902</v>
+      </c>
+      <c r="D42" t="n">
+        <v>4435192</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>73</v>
+      </c>
+      <c r="B43" t="n">
+        <v>3932235</v>
+      </c>
+      <c r="C43" t="n">
+        <v>25490185</v>
+      </c>
+      <c r="D43" t="n">
+        <v>4656952</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>74</v>
+      </c>
+      <c r="B44" t="n">
+        <v>3823527</v>
+      </c>
+      <c r="C44" t="n">
+        <v>24423912</v>
+      </c>
+      <c r="D44" t="n">
+        <v>4889800</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>75</v>
+      </c>
+      <c r="B45" t="n">
+        <v>3663586</v>
+      </c>
+      <c r="C45" t="n">
+        <v>22953208</v>
+      </c>
+      <c r="D45" t="n">
+        <v>5134290</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>76</v>
+      </c>
+      <c r="B46" t="n">
+        <v>3442981</v>
+      </c>
+      <c r="C46" t="n">
+        <v>21005185</v>
+      </c>
+      <c r="D46" t="n">
+        <v>5391004</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>77</v>
+      </c>
+      <c r="B47" t="n">
+        <v>3150777</v>
+      </c>
+      <c r="C47" t="n">
+        <v>18495408</v>
+      </c>
+      <c r="D47" t="n">
+        <v>5660554</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>78</v>
+      </c>
+      <c r="B48" t="n">
+        <v>2774311</v>
+      </c>
+      <c r="C48" t="n">
+        <v>15326137</v>
+      </c>
+      <c r="D48" t="n">
+        <v>5943582</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>79</v>
+      </c>
+      <c r="B49" t="n">
+        <v>2298920</v>
+      </c>
+      <c r="C49" t="n">
+        <v>11384296</v>
+      </c>
+      <c r="D49" t="n">
+        <v>6240761</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>80</v>
+      </c>
+      <c r="B50" t="n">
+        <v>1707644</v>
+      </c>
+      <c r="C50" t="n">
+        <v>6539141</v>
+      </c>
+      <c r="D50" t="n">
+        <v>6552799</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Migrate dashboard storage to Supabase
</commit_message>
<xml_diff>
--- a/static/annuitySchedule_results.xlsx
+++ b/static/annuitySchedule_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -440,13 +440,13 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>32</v>
+        <v>60</v>
       </c>
       <c r="B2" t="n">
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>6539011</v>
+        <v>35024487</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -454,674 +454,352 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="B3" t="n">
-        <v>980851</v>
+        <v>3852693</v>
       </c>
       <c r="C3" t="n">
-        <v>6858362</v>
+        <v>36284015</v>
       </c>
       <c r="D3" t="n">
-        <v>661500</v>
+        <v>2593165</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>34</v>
+        <v>62</v>
       </c>
       <c r="B4" t="n">
-        <v>1028754</v>
+        <v>3991241</v>
       </c>
       <c r="C4" t="n">
-        <v>7192541</v>
+        <v>37552433</v>
       </c>
       <c r="D4" t="n">
-        <v>694575</v>
+        <v>2722823</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>35</v>
+        <v>63</v>
       </c>
       <c r="B5" t="n">
-        <v>1078881</v>
+        <v>4130767</v>
       </c>
       <c r="C5" t="n">
-        <v>7542119</v>
+        <v>38824236</v>
       </c>
       <c r="D5" t="n">
-        <v>729303</v>
+        <v>2858964</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>36</v>
+        <v>64</v>
       </c>
       <c r="B6" t="n">
-        <v>1131317</v>
+        <v>4270665</v>
       </c>
       <c r="C6" t="n">
-        <v>7907668</v>
+        <v>40092989</v>
       </c>
       <c r="D6" t="n">
-        <v>765768</v>
+        <v>3001912</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>37</v>
+        <v>65</v>
       </c>
       <c r="B7" t="n">
-        <v>1186150</v>
+        <v>4410228</v>
       </c>
       <c r="C7" t="n">
-        <v>8289761</v>
+        <v>41351209</v>
       </c>
       <c r="D7" t="n">
-        <v>804057</v>
+        <v>3152008</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>38</v>
+        <v>66</v>
       </c>
       <c r="B8" t="n">
-        <v>1243464</v>
+        <v>4548632</v>
       </c>
       <c r="C8" t="n">
-        <v>8688965</v>
+        <v>42590233</v>
       </c>
       <c r="D8" t="n">
-        <v>844260</v>
+        <v>3309608</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>39</v>
+        <v>67</v>
       </c>
       <c r="B9" t="n">
-        <v>1303344</v>
+        <v>4684925</v>
       </c>
       <c r="C9" t="n">
-        <v>9105836</v>
+        <v>43800069</v>
       </c>
       <c r="D9" t="n">
-        <v>886473</v>
+        <v>3475089</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>40</v>
+        <v>68</v>
       </c>
       <c r="B10" t="n">
-        <v>1365875</v>
+        <v>4818007</v>
       </c>
       <c r="C10" t="n">
-        <v>9540915</v>
+        <v>44969233</v>
       </c>
       <c r="D10" t="n">
-        <v>930796</v>
+        <v>3648843</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>41</v>
+        <v>69</v>
       </c>
       <c r="B11" t="n">
-        <v>1431137</v>
+        <v>4946615</v>
       </c>
       <c r="C11" t="n">
-        <v>9994716</v>
+        <v>46084563</v>
       </c>
       <c r="D11" t="n">
-        <v>977336</v>
+        <v>3831285</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>42</v>
+        <v>70</v>
       </c>
       <c r="B12" t="n">
-        <v>1499207</v>
+        <v>5069301</v>
       </c>
       <c r="C12" t="n">
-        <v>10467720</v>
+        <v>47131014</v>
       </c>
       <c r="D12" t="n">
-        <v>1026203</v>
+        <v>4022850</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>43</v>
+        <v>71</v>
       </c>
       <c r="B13" t="n">
-        <v>1570158</v>
+        <v>5184411</v>
       </c>
       <c r="C13" t="n">
-        <v>10960365</v>
+        <v>48091433</v>
       </c>
       <c r="D13" t="n">
-        <v>1077513</v>
+        <v>4223992</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>44</v>
+        <v>72</v>
       </c>
       <c r="B14" t="n">
-        <v>1644054</v>
+        <v>5290057</v>
       </c>
       <c r="C14" t="n">
-        <v>11473030</v>
+        <v>48946298</v>
       </c>
       <c r="D14" t="n">
-        <v>1131389</v>
+        <v>4435192</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>45</v>
+        <v>73</v>
       </c>
       <c r="B15" t="n">
-        <v>1720954</v>
+        <v>5384092</v>
       </c>
       <c r="C15" t="n">
-        <v>12006026</v>
+        <v>49673439</v>
       </c>
       <c r="D15" t="n">
-        <v>1187958</v>
+        <v>4656951</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>46</v>
+        <v>74</v>
       </c>
       <c r="B16" t="n">
-        <v>1800903</v>
+        <v>5464078</v>
       </c>
       <c r="C16" t="n">
-        <v>12559573</v>
+        <v>50247718</v>
       </c>
       <c r="D16" t="n">
-        <v>1247356</v>
+        <v>4889799</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>47</v>
+        <v>75</v>
       </c>
       <c r="B17" t="n">
-        <v>1883935</v>
+        <v>5527248</v>
       </c>
       <c r="C17" t="n">
-        <v>13133784</v>
+        <v>50640677</v>
       </c>
       <c r="D17" t="n">
-        <v>1309724</v>
+        <v>5134289</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>48</v>
+        <v>76</v>
       </c>
       <c r="B18" t="n">
-        <v>1970067</v>
+        <v>5570474</v>
       </c>
       <c r="C18" t="n">
-        <v>13728641</v>
+        <v>50820148</v>
       </c>
       <c r="D18" t="n">
-        <v>1375210</v>
+        <v>5391003</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>49</v>
+        <v>77</v>
       </c>
       <c r="B19" t="n">
-        <v>2059296</v>
+        <v>5590216</v>
       </c>
       <c r="C19" t="n">
-        <v>14343966</v>
+        <v>50749811</v>
       </c>
       <c r="D19" t="n">
-        <v>1443971</v>
+        <v>5660553</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>50</v>
+        <v>78</v>
       </c>
       <c r="B20" t="n">
-        <v>2151594</v>
+        <v>5582479</v>
       </c>
       <c r="C20" t="n">
-        <v>14979390</v>
+        <v>50388709</v>
       </c>
       <c r="D20" t="n">
-        <v>1516170</v>
+        <v>5943581</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>51</v>
+        <v>79</v>
       </c>
       <c r="B21" t="n">
-        <v>2246908</v>
+        <v>5542757</v>
       </c>
       <c r="C21" t="n">
-        <v>15634320</v>
+        <v>49690706</v>
       </c>
       <c r="D21" t="n">
-        <v>1591978</v>
+        <v>6240760</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>52</v>
+        <v>80</v>
       </c>
       <c r="B22" t="n">
-        <v>2345148</v>
+        <v>5465977</v>
       </c>
       <c r="C22" t="n">
-        <v>16307891</v>
+        <v>48603885</v>
       </c>
       <c r="D22" t="n">
-        <v>1671577</v>
+        <v>6552798</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>53</v>
+        <v>81</v>
       </c>
       <c r="B23" t="n">
-        <v>2446183</v>
+        <v>5346427</v>
       </c>
       <c r="C23" t="n">
-        <v>16998918</v>
+        <v>47069874</v>
       </c>
       <c r="D23" t="n">
-        <v>1755156</v>
+        <v>6880438</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>54</v>
+        <v>82</v>
       </c>
       <c r="B24" t="n">
-        <v>2549837</v>
+        <v>5177686</v>
       </c>
       <c r="C24" t="n">
-        <v>17705841</v>
+        <v>45023100</v>
       </c>
       <c r="D24" t="n">
-        <v>1842914</v>
+        <v>7224460</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>55</v>
+        <v>83</v>
       </c>
       <c r="B25" t="n">
-        <v>2655876</v>
+        <v>4952541</v>
       </c>
       <c r="C25" t="n">
-        <v>18426658</v>
+        <v>42389958</v>
       </c>
       <c r="D25" t="n">
-        <v>1935059</v>
+        <v>7585683</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>56</v>
+        <v>84</v>
       </c>
       <c r="B26" t="n">
-        <v>2763998</v>
+        <v>4662895</v>
       </c>
       <c r="C26" t="n">
-        <v>19158844</v>
+        <v>39087886</v>
       </c>
       <c r="D26" t="n">
-        <v>2031812</v>
+        <v>7964967</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>57</v>
+        <v>85</v>
       </c>
       <c r="B27" t="n">
-        <v>2873826</v>
+        <v>4299667</v>
       </c>
       <c r="C27" t="n">
-        <v>19899267</v>
+        <v>35024337</v>
       </c>
       <c r="D27" t="n">
-        <v>2133403</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>58</v>
-      </c>
-      <c r="B28" t="n">
-        <v>2984890</v>
-      </c>
-      <c r="C28" t="n">
-        <v>20644084</v>
-      </c>
-      <c r="D28" t="n">
-        <v>2240073</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>59</v>
-      </c>
-      <c r="B29" t="n">
-        <v>3096612</v>
-      </c>
-      <c r="C29" t="n">
-        <v>21388619</v>
-      </c>
-      <c r="D29" t="n">
-        <v>2352077</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>60</v>
-      </c>
-      <c r="B30" t="n">
-        <v>3208292</v>
-      </c>
-      <c r="C30" t="n">
-        <v>22127230</v>
-      </c>
-      <c r="D30" t="n">
-        <v>2469681</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>61</v>
-      </c>
-      <c r="B31" t="n">
-        <v>3319084</v>
-      </c>
-      <c r="C31" t="n">
-        <v>22853149</v>
-      </c>
-      <c r="D31" t="n">
-        <v>2593165</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>62</v>
-      </c>
-      <c r="B32" t="n">
-        <v>3427972</v>
-      </c>
-      <c r="C32" t="n">
-        <v>23558298</v>
-      </c>
-      <c r="D32" t="n">
-        <v>2722823</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>63</v>
-      </c>
-      <c r="B33" t="n">
-        <v>3533744</v>
-      </c>
-      <c r="C33" t="n">
-        <v>24233078</v>
-      </c>
-      <c r="D33" t="n">
-        <v>2858964</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="n">
-        <v>64</v>
-      </c>
-      <c r="B34" t="n">
-        <v>3634961</v>
-      </c>
-      <c r="C34" t="n">
-        <v>24866126</v>
-      </c>
-      <c r="D34" t="n">
-        <v>3001913</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="n">
-        <v>65</v>
-      </c>
-      <c r="B35" t="n">
-        <v>3729918</v>
-      </c>
-      <c r="C35" t="n">
-        <v>25444036</v>
-      </c>
-      <c r="D35" t="n">
-        <v>3152008</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>66</v>
-      </c>
-      <c r="B36" t="n">
-        <v>3816605</v>
-      </c>
-      <c r="C36" t="n">
-        <v>25951032</v>
-      </c>
-      <c r="D36" t="n">
-        <v>3309609</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="n">
-        <v>67</v>
-      </c>
-      <c r="B37" t="n">
-        <v>3892654</v>
-      </c>
-      <c r="C37" t="n">
-        <v>26368597</v>
-      </c>
-      <c r="D37" t="n">
-        <v>3475089</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="n">
-        <v>68</v>
-      </c>
-      <c r="B38" t="n">
-        <v>3955289</v>
-      </c>
-      <c r="C38" t="n">
-        <v>26675042</v>
-      </c>
-      <c r="D38" t="n">
-        <v>3648844</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="n">
-        <v>69</v>
-      </c>
-      <c r="B39" t="n">
-        <v>4001256</v>
-      </c>
-      <c r="C39" t="n">
-        <v>26845012</v>
-      </c>
-      <c r="D39" t="n">
-        <v>3831286</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="n">
-        <v>70</v>
-      </c>
-      <c r="B40" t="n">
-        <v>4026751</v>
-      </c>
-      <c r="C40" t="n">
-        <v>26848913</v>
-      </c>
-      <c r="D40" t="n">
-        <v>4022850</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="n">
-        <v>71</v>
-      </c>
-      <c r="B41" t="n">
-        <v>4027336</v>
-      </c>
-      <c r="C41" t="n">
-        <v>26652256</v>
-      </c>
-      <c r="D41" t="n">
-        <v>4223993</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="n">
-        <v>72</v>
-      </c>
-      <c r="B42" t="n">
-        <v>3997838</v>
-      </c>
-      <c r="C42" t="n">
-        <v>26214902</v>
-      </c>
-      <c r="D42" t="n">
-        <v>4435192</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>73</v>
-      </c>
-      <c r="B43" t="n">
-        <v>3932235</v>
-      </c>
-      <c r="C43" t="n">
-        <v>25490185</v>
-      </c>
-      <c r="D43" t="n">
-        <v>4656952</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
-        <v>74</v>
-      </c>
-      <c r="B44" t="n">
-        <v>3823527</v>
-      </c>
-      <c r="C44" t="n">
-        <v>24423912</v>
-      </c>
-      <c r="D44" t="n">
-        <v>4889800</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="n">
-        <v>75</v>
-      </c>
-      <c r="B45" t="n">
-        <v>3663586</v>
-      </c>
-      <c r="C45" t="n">
-        <v>22953208</v>
-      </c>
-      <c r="D45" t="n">
-        <v>5134290</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="n">
-        <v>76</v>
-      </c>
-      <c r="B46" t="n">
-        <v>3442981</v>
-      </c>
-      <c r="C46" t="n">
-        <v>21005185</v>
-      </c>
-      <c r="D46" t="n">
-        <v>5391004</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="n">
-        <v>77</v>
-      </c>
-      <c r="B47" t="n">
-        <v>3150777</v>
-      </c>
-      <c r="C47" t="n">
-        <v>18495408</v>
-      </c>
-      <c r="D47" t="n">
-        <v>5660554</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="n">
-        <v>78</v>
-      </c>
-      <c r="B48" t="n">
-        <v>2774311</v>
-      </c>
-      <c r="C48" t="n">
-        <v>15326137</v>
-      </c>
-      <c r="D48" t="n">
-        <v>5943582</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="n">
-        <v>79</v>
-      </c>
-      <c r="B49" t="n">
-        <v>2298920</v>
-      </c>
-      <c r="C49" t="n">
-        <v>11384296</v>
-      </c>
-      <c r="D49" t="n">
-        <v>6240761</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="n">
-        <v>80</v>
-      </c>
-      <c r="B50" t="n">
-        <v>1707644</v>
-      </c>
-      <c r="C50" t="n">
-        <v>6539141</v>
-      </c>
-      <c r="D50" t="n">
-        <v>6552799</v>
+        <v>8363216</v>
       </c>
     </row>
   </sheetData>

</xml_diff>